<commit_message>
Adjust 23 Jul to 10-6 roster and close at 22:00.
Align day to 10:00-18:00 with lunch 14:00-14:30 and log beyond-hours work through 22:00.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/exports/FlightPath_Daily_Work_2026-07-23.xlsx
+++ b/exports/FlightPath_Daily_Work_2026-07-23.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Day Rollup" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02 Daily Log'!$A$1:$L$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02 Daily Log'!$A$1:$L$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04 Day Rollup'!$A$1:$I$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -61,7 +61,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -76,6 +76,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F4F7F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -105,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -125,6 +130,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -448,8 +456,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DailyLog" displayName="DailyLog" ref="A1:L5" headerRowCount="1">
-  <autoFilter ref="A1:L5"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DailyLog" displayName="DailyLog" ref="A1:L6" headerRowCount="1">
+  <autoFilter ref="A1:L6"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Date"/>
     <tableColumn id="2" name="Weekday"/>
@@ -870,10 +878,10 @@
         </is>
       </c>
       <c r="E5" s="6" t="n">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
@@ -884,10 +892,10 @@
         <v>1</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -897,7 +905,7 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>8</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="7">
@@ -907,7 +915,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -937,7 +945,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>8</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="11"/>
@@ -967,21 +975,21 @@
     <row r="15">
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Team Support</t>
+          <t>Internal Tools</t>
         </is>
       </c>
       <c r="E15" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16">
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>Internal Tools</t>
+          <t>Team Support</t>
         </is>
       </c>
       <c r="E16" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17">
@@ -991,7 +999,7 @@
         </is>
       </c>
       <c r="E17" s="6" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="18"/>
@@ -1237,7 +1245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1349,12 +1357,12 @@
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="I2" s="5" t="n">
@@ -1409,12 +1417,12 @@
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="I3" s="5" t="n">
@@ -1469,12 +1477,12 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="I4" s="5" t="n">
@@ -1529,16 +1537,16 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
@@ -1556,8 +1564,68 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>HR assigned + Flipkart suite / platform</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Internal Tools</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="J6" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K6" s="11" t="inlineStr">
+        <is>
+          <t>Complete daily task update with agent</t>
+        </is>
+      </c>
+      <c r="L6" s="11" t="inlineStr">
+        <is>
+          <t>Closed today’s work log / tracker update with Cursor agent; complete at ~22:00.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L5"/>
+  <autoFilter ref="A1:L6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1642,13 +1710,13 @@
         <v>0</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>8</v>
+        <v>11.5</v>
       </c>
       <c r="H2" s="5" t="n">
         <v>30</v>
@@ -1676,7 +1744,7 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="31" customWidth="1" min="9" max="9"/>
+    <col width="39" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1753,17 +1821,17 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Laptop asset purchase support</t>
+          <t>Complete daily task update with agent</t>
         </is>
       </c>
     </row>

</xml_diff>